<commit_message>
Update Dexcom job tracker
</commit_message>
<xml_diff>
--- a/Dexcom_Job_Tracker.xlsx
+++ b/Dexcom_Job_Tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Dexcom Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dexcom Job Tracker'!$A$1:$D$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dexcom Job Tracker'!$A$1:$D$179</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -95,6 +95,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -635,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D157"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -667,12 +676,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="57" t="inlineStr">
+      <c r="A2" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B2" s="58" t="n">
+      <c r="B2" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -680,19 +689,19 @@
           <t>Associate Facilities Engineer (Building Maintenance)</t>
         </is>
       </c>
-      <c r="D2" s="59" t="inlineStr">
+      <c r="D2" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4459144568/</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="57" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="B3" s="58" t="n">
+      <c r="B3" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -700,19 +709,19 @@
           <t>Executive Assistant - Madrid</t>
         </is>
       </c>
-      <c r="D3" s="59" t="inlineStr">
+      <c r="D3" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4448303180/</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="57" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B4" s="58" t="n">
+      <c r="B4" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -720,19 +729,19 @@
           <t>Benefits Analyst</t>
         </is>
       </c>
-      <c r="D4" s="59" t="inlineStr">
+      <c r="D4" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4461581171/</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="57" t="inlineStr">
+      <c r="A5" s="60" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="B5" s="58" t="n">
+      <c r="B5" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -740,19 +749,19 @@
           <t>Senior Manager Corporate Compliance - EMEA</t>
         </is>
       </c>
-      <c r="D5" s="59" t="inlineStr">
+      <c r="D5" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4429707112/</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="57" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B6" s="58" t="n">
+      <c r="B6" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -760,19 +769,19 @@
           <t>Customer Service Representative (German-speaking)</t>
         </is>
       </c>
-      <c r="D6" s="59" t="inlineStr">
+      <c r="D6" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4463120173/</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="57" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B7" s="58" t="n">
+      <c r="B7" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -780,19 +789,19 @@
           <t>Sr Enterprise Privacy Analyst</t>
         </is>
       </c>
-      <c r="D7" s="59" t="inlineStr">
+      <c r="D7" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4387414194/</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="57" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B8" s="58" t="n">
+      <c r="B8" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -800,19 +809,19 @@
           <t>Customer Advocacy Generalist</t>
         </is>
       </c>
-      <c r="D8" s="59" t="inlineStr">
+      <c r="D8" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4461765131/</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="57" t="inlineStr">
+      <c r="A9" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B9" s="58" t="n">
+      <c r="B9" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -820,19 +829,19 @@
           <t>Customer Advocacy Generalist</t>
         </is>
       </c>
-      <c r="D9" s="59" t="inlineStr">
+      <c r="D9" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4459303523/</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="57" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B10" s="58" t="n">
+      <c r="B10" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -840,19 +849,19 @@
           <t>Associate Facilities Engineer</t>
         </is>
       </c>
-      <c r="D10" s="59" t="inlineStr">
+      <c r="D10" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4448830718/</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="57" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B11" s="58" t="n">
+      <c r="B11" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -860,19 +869,19 @@
           <t>Sr Cybersecurity Analyst - GRC</t>
         </is>
       </c>
-      <c r="D11" s="59" t="inlineStr">
+      <c r="D11" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4454019825/</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="57" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B12" s="58" t="n">
+      <c r="B12" s="61" t="n">
         <v>46276</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -880,19 +889,19 @@
           <t>Sr Manager Human Resources</t>
         </is>
       </c>
-      <c r="D12" s="59" t="inlineStr">
+      <c r="D12" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4466052473/</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="57" t="inlineStr">
+      <c r="A13" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B13" s="58" t="n">
+      <c r="B13" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -900,19 +909,19 @@
           <t>Sr. Manager - Capability Leader, Sentiment Intelligence</t>
         </is>
       </c>
-      <c r="D13" s="59" t="inlineStr">
+      <c r="D13" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4459302533/</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="57" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B14" s="58" t="n">
+      <c r="B14" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -920,19 +929,19 @@
           <t>Sr Cost Accountant</t>
         </is>
       </c>
-      <c r="D14" s="59" t="inlineStr">
+      <c r="D14" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4410011461/</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="57" t="inlineStr">
+      <c r="A15" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B15" s="58" t="n">
+      <c r="B15" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -940,19 +949,19 @@
           <t>Sr Regulatory Affairs Specialist</t>
         </is>
       </c>
-      <c r="D15" s="59" t="inlineStr">
+      <c r="D15" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4448601784/</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="57" t="inlineStr">
+      <c r="A16" s="60" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B16" s="58" t="n">
+      <c r="B16" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -960,19 +969,19 @@
           <t>Software Development Engineer 2</t>
         </is>
       </c>
-      <c r="D16" s="59" t="inlineStr">
+      <c r="D16" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453360435/</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="57" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B17" s="58" t="n">
+      <c r="B17" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -980,19 +989,19 @@
           <t>Sr Facilities Engineer</t>
         </is>
       </c>
-      <c r="D17" s="59" t="inlineStr">
+      <c r="D17" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4446562908/</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="57" t="inlineStr">
+      <c r="A18" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B18" s="58" t="n">
+      <c r="B18" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1000,19 +1009,19 @@
           <t>Sr Cybersecurity Analyst - GRC</t>
         </is>
       </c>
-      <c r="D18" s="59" t="inlineStr">
+      <c r="D18" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453096131/</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="57" t="inlineStr">
+      <c r="A19" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B19" s="58" t="n">
+      <c r="B19" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1020,19 +1029,19 @@
           <t>Accountant - Healthcare - Edinburgh</t>
         </is>
       </c>
-      <c r="D19" s="59" t="inlineStr">
+      <c r="D19" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453144035/</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="57" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="B20" s="58" t="n">
+      <c r="B20" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1040,19 +1049,19 @@
           <t>Manager Finance</t>
         </is>
       </c>
-      <c r="D20" s="59" t="inlineStr">
+      <c r="D20" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4462145294/</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="57" t="inlineStr">
+      <c r="A21" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B21" s="58" t="n">
+      <c r="B21" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1060,19 +1069,19 @@
           <t>Regulatory Affairs Specialist</t>
         </is>
       </c>
-      <c r="D21" s="59" t="inlineStr">
+      <c r="D21" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4448398864/</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="57" t="inlineStr">
+      <c r="A22" s="60" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="B22" s="58" t="n">
+      <c r="B22" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1080,19 +1089,19 @@
           <t>Senior Manager Corporate Compliance - EMEA (m/w/d)</t>
         </is>
       </c>
-      <c r="D22" s="59" t="inlineStr">
+      <c r="D22" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4461752409/</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="57" t="inlineStr">
+      <c r="A23" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B23" s="58" t="n">
+      <c r="B23" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1100,19 +1109,19 @@
           <t>Director, QA - Product Development Processes</t>
         </is>
       </c>
-      <c r="D23" s="59" t="inlineStr">
+      <c r="D23" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4456434433/</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="57" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B24" s="58" t="n">
+      <c r="B24" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1120,19 +1129,19 @@
           <t>Security and Privacy Compliance Analyst - Cybersecurity</t>
         </is>
       </c>
-      <c r="D24" s="59" t="inlineStr">
+      <c r="D24" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4257269392/</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="57" t="inlineStr">
+      <c r="A25" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B25" s="58" t="n">
+      <c r="B25" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1140,19 +1149,19 @@
           <t>Advanced Support Specialist 1</t>
         </is>
       </c>
-      <c r="D25" s="59" t="inlineStr">
+      <c r="D25" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4458769459/</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="57" t="inlineStr">
+      <c r="A26" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B26" s="58" t="n">
+      <c r="B26" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -1160,19 +1169,19 @@
           <t>Sr Quality Assurance Analyst</t>
         </is>
       </c>
-      <c r="D26" s="59" t="inlineStr">
+      <c r="D26" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4451545592/</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="57" t="inlineStr">
+      <c r="A27" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B27" s="58" t="n">
+      <c r="B27" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1180,19 +1189,19 @@
           <t>Sr. Manager-Vendor Management (Electronics)</t>
         </is>
       </c>
-      <c r="D27" s="59" t="inlineStr">
+      <c r="D27" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4446726237/</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="57" t="inlineStr">
+      <c r="A28" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B28" s="58" t="n">
+      <c r="B28" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -1200,19 +1209,19 @@
           <t>Customer Success Associate</t>
         </is>
       </c>
-      <c r="D28" s="59" t="inlineStr">
+      <c r="D28" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4447526678/</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="57" t="inlineStr">
+      <c r="A29" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B29" s="58" t="n">
+      <c r="B29" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -1220,19 +1229,19 @@
           <t>Supply Chain Analyst</t>
         </is>
       </c>
-      <c r="D29" s="59" t="inlineStr">
+      <c r="D29" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4433857606/</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="57" t="inlineStr">
+      <c r="A30" s="60" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="B30" s="58" t="n">
+      <c r="B30" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -1240,19 +1249,19 @@
           <t>Manager, APAC Business Development and Partnership</t>
         </is>
       </c>
-      <c r="D30" s="59" t="inlineStr">
+      <c r="D30" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453097086/</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="57" t="inlineStr">
+      <c r="A31" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B31" s="58" t="n">
+      <c r="B31" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -1260,19 +1269,19 @@
           <t>Sr Quality Engineer, Supplier Quality Engineering</t>
         </is>
       </c>
-      <c r="D31" s="59" t="inlineStr">
+      <c r="D31" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4384568916/</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="57" t="inlineStr">
+      <c r="A32" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B32" s="58" t="n">
+      <c r="B32" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -1280,19 +1289,19 @@
           <t>Sr QA Engineer</t>
         </is>
       </c>
-      <c r="D32" s="59" t="inlineStr">
+      <c r="D32" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4465859501/</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="57" t="inlineStr">
+      <c r="A33" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B33" s="58" t="n">
+      <c r="B33" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -1300,19 +1309,19 @@
           <t>Staff Data Engineer</t>
         </is>
       </c>
-      <c r="D33" s="59" t="inlineStr">
+      <c r="D33" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4446368700/</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="57" t="inlineStr">
+      <c r="A34" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B34" s="58" t="n">
+      <c r="B34" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -1320,19 +1329,19 @@
           <t>Senior Sustainability Specialist – Healthcare – Vilnius, Lithuania</t>
         </is>
       </c>
-      <c r="D34" s="59" t="inlineStr">
+      <c r="D34" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4459828416/</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="57" t="inlineStr">
+      <c r="A35" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B35" s="58" t="n">
+      <c r="B35" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -1340,19 +1349,19 @@
           <t>Associate Territory Sales Manager - Healthcare - Leicestershire &amp; Lincolnshire</t>
         </is>
       </c>
-      <c r="D35" s="59" t="inlineStr">
+      <c r="D35" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453077256/</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="57" t="inlineStr">
+      <c r="A36" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B36" s="58" t="n">
+      <c r="B36" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -1360,19 +1369,19 @@
           <t>Manager, APAC Business Development and Partnership</t>
         </is>
       </c>
-      <c r="D36" s="59" t="inlineStr">
+      <c r="D36" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453093132/</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="57" t="inlineStr">
+      <c r="A37" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B37" s="58" t="n">
+      <c r="B37" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -1380,19 +1389,19 @@
           <t>Sr Systems Engineer</t>
         </is>
       </c>
-      <c r="D37" s="59" t="inlineStr">
+      <c r="D37" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4371263716/</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="57" t="inlineStr">
+      <c r="A38" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B38" s="58" t="n">
+      <c r="B38" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -1400,19 +1409,19 @@
           <t>Customer Service Representative - French Speaker</t>
         </is>
       </c>
-      <c r="D38" s="59" t="inlineStr">
+      <c r="D38" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4460500502/</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="57" t="inlineStr">
+      <c r="A39" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B39" s="58" t="n">
+      <c r="B39" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -1420,19 +1429,19 @@
           <t>Program Manager - AI Initiatives</t>
         </is>
       </c>
-      <c r="D39" s="59" t="inlineStr">
+      <c r="D39" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4435119512/</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="57" t="inlineStr">
+      <c r="A40" s="60" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="B40" s="58" t="n">
+      <c r="B40" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -1440,19 +1449,19 @@
           <t>Sr Sales Trainer Diabetes MEA</t>
         </is>
       </c>
-      <c r="D40" s="59" t="inlineStr">
+      <c r="D40" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4449635545/</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="57" t="inlineStr">
+      <c r="A41" s="60" t="inlineStr">
         <is>
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="B41" s="58" t="n">
+      <c r="B41" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -1460,19 +1469,19 @@
           <t>Territory Sales Manager (m/w/d) - Zentralschweiz : Luzern, Obwalden, Nidwalden, Uri, Chur</t>
         </is>
       </c>
-      <c r="D41" s="59" t="inlineStr">
+      <c r="D41" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453133160/</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="57" t="inlineStr">
+      <c r="A42" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B42" s="58" t="n">
+      <c r="B42" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -1480,19 +1489,19 @@
           <t>Speaker Bureau and KOL Operations Manager</t>
         </is>
       </c>
-      <c r="D42" s="59" t="inlineStr">
+      <c r="D42" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4423312162/</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="57" t="inlineStr">
+      <c r="A43" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B43" s="58" t="n">
+      <c r="B43" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -1500,19 +1509,19 @@
           <t>Process Development Engineer 2</t>
         </is>
       </c>
-      <c r="D43" s="59" t="inlineStr">
+      <c r="D43" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4437873233/</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="57" t="inlineStr">
+      <c r="A44" s="60" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="B44" s="58" t="n">
+      <c r="B44" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -1520,19 +1529,19 @@
           <t>Marketing Manager Education Consumer Products EMEA – Healthcare – Barcelona, Spain</t>
         </is>
       </c>
-      <c r="D44" s="59" t="inlineStr">
+      <c r="D44" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4459811610/</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="57" t="inlineStr">
+      <c r="A45" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B45" s="58" t="n">
+      <c r="B45" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -1540,19 +1549,19 @@
           <t>Technical Support Representative 1</t>
         </is>
       </c>
-      <c r="D45" s="59" t="inlineStr">
+      <c r="D45" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4403461287/</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="57" t="inlineStr">
+      <c r="A46" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B46" s="58" t="n">
+      <c r="B46" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -1560,19 +1569,19 @@
           <t>Sr Manager Regulatory Affairs- LATAM</t>
         </is>
       </c>
-      <c r="D46" s="59" t="inlineStr">
+      <c r="D46" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4448606739/</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="57" t="inlineStr">
+      <c r="A47" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B47" s="58" t="n">
+      <c r="B47" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -1580,19 +1589,19 @@
           <t>Associate Territory Sales Manager - Healthcare - Leicestershire &amp; Lincolnshire</t>
         </is>
       </c>
-      <c r="D47" s="59" t="inlineStr">
+      <c r="D47" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453075275/</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="57" t="inlineStr">
+      <c r="A48" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B48" s="58" t="n">
+      <c r="B48" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -1600,19 +1609,19 @@
           <t>Customer Account Support Specialist 2</t>
         </is>
       </c>
-      <c r="D48" s="59" t="inlineStr">
+      <c r="D48" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4450027435/</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="57" t="inlineStr">
+      <c r="A49" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B49" s="58" t="n">
+      <c r="B49" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -1620,19 +1629,19 @@
           <t>Procurement Ops Manager (IC)</t>
         </is>
       </c>
-      <c r="D49" s="59" t="inlineStr">
+      <c r="D49" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453097103/</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="57" t="inlineStr">
+      <c r="A50" s="60" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B50" s="58" t="n">
+      <c r="B50" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -1640,19 +1649,19 @@
           <t>Senior Software Development Engineer</t>
         </is>
       </c>
-      <c r="D50" s="59" t="inlineStr">
+      <c r="D50" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453371096/</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="57" t="inlineStr">
+      <c r="A51" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B51" s="58" t="n">
+      <c r="B51" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -1660,19 +1669,19 @@
           <t>Technical Support Representative 1</t>
         </is>
       </c>
-      <c r="D51" s="59" t="inlineStr">
+      <c r="D51" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4403153694/</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="57" t="inlineStr">
+      <c r="A52" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B52" s="58" t="n">
+      <c r="B52" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -1680,19 +1689,19 @@
           <t>Junior Territory Sales Manager - Healthcare - Hertfordshire &amp; Essex</t>
         </is>
       </c>
-      <c r="D52" s="59" t="inlineStr">
+      <c r="D52" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453092177/</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="57" t="inlineStr">
+      <c r="A53" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B53" s="58" t="n">
+      <c r="B53" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -1700,19 +1709,19 @@
           <t>Graphic Designer 2</t>
         </is>
       </c>
-      <c r="D53" s="59" t="inlineStr">
+      <c r="D53" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4456722826/</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="57" t="inlineStr">
+      <c r="A54" s="60" t="inlineStr">
         <is>
           <t>Ireland</t>
         </is>
       </c>
-      <c r="B54" s="58" t="n">
+      <c r="B54" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -1720,19 +1729,19 @@
           <t>Purchasing Manager</t>
         </is>
       </c>
-      <c r="D54" s="59" t="inlineStr">
+      <c r="D54" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4458283492/</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="57" t="inlineStr">
+      <c r="A55" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B55" s="58" t="n">
+      <c r="B55" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -1740,19 +1749,19 @@
           <t>Manufacturing Associate 2</t>
         </is>
       </c>
-      <c r="D55" s="59" t="inlineStr">
+      <c r="D55" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4456472809/</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="57" t="inlineStr">
+      <c r="A56" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B56" s="58" t="n">
+      <c r="B56" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -1760,19 +1769,19 @@
           <t>Engineering Technician 2</t>
         </is>
       </c>
-      <c r="D56" s="59" t="inlineStr">
+      <c r="D56" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4465624957/</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="57" t="inlineStr">
+      <c r="A57" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B57" s="58" t="n">
+      <c r="B57" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -1780,19 +1789,19 @@
           <t>Engineering Technician 4</t>
         </is>
       </c>
-      <c r="D57" s="59" t="inlineStr">
+      <c r="D57" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4438139166/</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="57" t="inlineStr">
+      <c r="A58" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B58" s="58" t="n">
+      <c r="B58" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -1800,19 +1809,19 @@
           <t>Sr Cybersecurity Engineer</t>
         </is>
       </c>
-      <c r="D58" s="59" t="inlineStr">
+      <c r="D58" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4394381237/</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="57" t="inlineStr">
+      <c r="A59" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B59" s="58" t="n">
+      <c r="B59" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -1820,19 +1829,19 @@
           <t>Sr. Director, Consumer Software Applications</t>
         </is>
       </c>
-      <c r="D59" s="59" t="inlineStr">
+      <c r="D59" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4456361869/</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="57" t="inlineStr">
+      <c r="A60" s="60" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="B60" s="58" t="n">
+      <c r="B60" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -1840,19 +1849,19 @@
           <t>Kundenservice Medizintechnik (m/w/d) - Mainz</t>
         </is>
       </c>
-      <c r="D60" s="59" t="inlineStr">
+      <c r="D60" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4462192923/</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="57" t="inlineStr">
+      <c r="A61" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B61" s="58" t="n">
+      <c r="B61" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -1860,19 +1869,19 @@
           <t>Global Brand Marketing Manager (Stelo)</t>
         </is>
       </c>
-      <c r="D61" s="59" t="inlineStr">
+      <c r="D61" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4435306708/</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="57" t="inlineStr">
+      <c r="A62" s="60" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B62" s="58" t="n">
+      <c r="B62" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -1880,19 +1889,19 @@
           <t>Business Development Lead - India (Multiple Locations)</t>
         </is>
       </c>
-      <c r="D62" s="59" t="inlineStr">
+      <c r="D62" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4456463987/</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="57" t="inlineStr">
+      <c r="A63" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B63" s="58" t="n">
+      <c r="B63" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -1900,19 +1909,19 @@
           <t>Sr Manager Medical Affairs</t>
         </is>
       </c>
-      <c r="D63" s="59" t="inlineStr">
+      <c r="D63" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4461536483/</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="57" t="inlineStr">
+      <c r="A64" s="60" t="inlineStr">
         <is>
           <t>Ireland</t>
         </is>
       </c>
-      <c r="B64" s="58" t="n">
+      <c r="B64" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -1920,19 +1929,19 @@
           <t>Manufacturing Technician 3 (Weekend Day Shift)</t>
         </is>
       </c>
-      <c r="D64" s="59" t="inlineStr">
+      <c r="D64" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4456731799/</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="57" t="inlineStr">
+      <c r="A65" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B65" s="58" t="n">
+      <c r="B65" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -1940,19 +1949,19 @@
           <t>Staff Membrane Formulation Scientist</t>
         </is>
       </c>
-      <c r="D65" s="59" t="inlineStr">
+      <c r="D65" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4438128497/</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="57" t="inlineStr">
+      <c r="A66" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B66" s="58" t="n">
+      <c r="B66" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -1960,19 +1969,19 @@
           <t>Talent Acquisition Advisor (Maternity cover)</t>
         </is>
       </c>
-      <c r="D66" s="59" t="inlineStr">
+      <c r="D66" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4459039247/</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="57" t="inlineStr">
+      <c r="A67" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B67" s="58" t="n">
+      <c r="B67" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -1980,19 +1989,19 @@
           <t>Hardware Engineer 2</t>
         </is>
       </c>
-      <c r="D67" s="59" t="inlineStr">
+      <c r="D67" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4457567279/</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="57" t="inlineStr">
+      <c r="A68" s="60" t="inlineStr">
         <is>
           <t>Ireland</t>
         </is>
       </c>
-      <c r="B68" s="58" t="n">
+      <c r="B68" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -2000,19 +2009,19 @@
           <t>Senior Warehouse Operative - Weekend Days</t>
         </is>
       </c>
-      <c r="D68" s="59" t="inlineStr">
+      <c r="D68" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4461098658/</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="57" t="inlineStr">
+      <c r="A69" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B69" s="58" t="n">
+      <c r="B69" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -2020,19 +2029,19 @@
           <t>Junior Territory Sales Manager - Healthcare - Hertfordshire &amp; Essex</t>
         </is>
       </c>
-      <c r="D69" s="59" t="inlineStr">
+      <c r="D69" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453087192/</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="57" t="inlineStr">
+      <c r="A70" s="60" t="inlineStr">
         <is>
           <t>Slovenia</t>
         </is>
       </c>
-      <c r="B70" s="58" t="n">
+      <c r="B70" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -2040,19 +2049,19 @@
           <t>Sr Market Access Manager</t>
         </is>
       </c>
-      <c r="D70" s="59" t="inlineStr">
+      <c r="D70" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4465675855/</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="57" t="inlineStr">
+      <c r="A71" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B71" s="58" t="n">
+      <c r="B71" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -2060,19 +2069,19 @@
           <t>Marketing Manager Education Consumer Products EMEA – Healthcare – Barcelona, Spain</t>
         </is>
       </c>
-      <c r="D71" s="59" t="inlineStr">
+      <c r="D71" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4459816548/</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="57" t="inlineStr">
+      <c r="A72" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B72" s="58" t="n">
+      <c r="B72" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -2080,19 +2089,19 @@
           <t>Customer Advocacy Generalist</t>
         </is>
       </c>
-      <c r="D72" s="59" t="inlineStr">
+      <c r="D72" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4464354416/</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="57" t="inlineStr">
+      <c r="A73" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B73" s="58" t="n">
+      <c r="B73" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -2100,19 +2109,19 @@
           <t>Customer Advocacy Generalist</t>
         </is>
       </c>
-      <c r="D73" s="59" t="inlineStr">
+      <c r="D73" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4464339507/</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="57" t="inlineStr">
+      <c r="A74" s="60" t="inlineStr">
         <is>
           <t>Ireland</t>
         </is>
       </c>
-      <c r="B74" s="58" t="n">
+      <c r="B74" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -2120,19 +2129,19 @@
           <t>Senior QA Manager (Quality Systems)</t>
         </is>
       </c>
-      <c r="D74" s="59" t="inlineStr">
+      <c r="D74" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4457509031/</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="57" t="inlineStr">
+      <c r="A75" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B75" s="58" t="n">
+      <c r="B75" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -2140,19 +2149,19 @@
           <t>Customer Service Representative (Italian-speaking)</t>
         </is>
       </c>
-      <c r="D75" s="59" t="inlineStr">
+      <c r="D75" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4446389046/</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="57" t="inlineStr">
+      <c r="A76" s="60" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="B76" s="58" t="n">
+      <c r="B76" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -2160,19 +2169,19 @@
           <t>Senior Forecasting Analyst</t>
         </is>
       </c>
-      <c r="D76" s="59" t="inlineStr">
+      <c r="D76" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4463637144/</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="57" t="inlineStr">
+      <c r="A77" s="60" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="B77" s="58" t="n">
+      <c r="B77" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -2180,19 +2189,19 @@
           <t>Sales/Inside Sales Trainer - Healthcare (m/w/d)</t>
         </is>
       </c>
-      <c r="D77" s="59" t="inlineStr">
+      <c r="D77" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4461765129/</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="57" t="inlineStr">
+      <c r="A78" s="60" t="inlineStr">
         <is>
           <t>Ireland</t>
         </is>
       </c>
-      <c r="B78" s="58" t="n">
+      <c r="B78" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -2200,19 +2209,19 @@
           <t>Quality Technician 2 Back End Days</t>
         </is>
       </c>
-      <c r="D78" s="59" t="inlineStr">
+      <c r="D78" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4464613132/</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="57" t="inlineStr">
+      <c r="A79" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B79" s="58" t="n">
+      <c r="B79" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -2220,19 +2229,19 @@
           <t>Mitarbeiter:innen für den deutschsprachigen Produkt- und Kundendienst (m/w/d)</t>
         </is>
       </c>
-      <c r="D79" s="59" t="inlineStr">
+      <c r="D79" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4446570417/</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="57" t="inlineStr">
+      <c r="A80" s="60" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="B80" s="58" t="n">
+      <c r="B80" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -2240,19 +2249,19 @@
           <t>Senior Forecasting Analyst</t>
         </is>
       </c>
-      <c r="D80" s="59" t="inlineStr">
+      <c r="D80" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4463633190/</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="57" t="inlineStr">
+      <c r="A81" s="60" t="inlineStr">
         <is>
           <t>Italy</t>
         </is>
       </c>
-      <c r="B81" s="58" t="n">
+      <c r="B81" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -2260,19 +2269,19 @@
           <t>Sr Technical Program Manager FHIR APIs- 18 months fixed term</t>
         </is>
       </c>
-      <c r="D81" s="59" t="inlineStr">
+      <c r="D81" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4450696746/</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="57" t="inlineStr">
+      <c r="A82" s="60" t="inlineStr">
         <is>
           <t>Ireland</t>
         </is>
       </c>
-      <c r="B82" s="58" t="n">
+      <c r="B82" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -2280,19 +2289,19 @@
           <t>Logistics Analyst</t>
         </is>
       </c>
-      <c r="D82" s="59" t="inlineStr">
+      <c r="D82" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4461266744/</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="57" t="inlineStr">
+      <c r="A83" s="60" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="B83" s="58" t="n">
+      <c r="B83" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -2300,19 +2309,19 @@
           <t>Senior Forecasting Analyst</t>
         </is>
       </c>
-      <c r="D83" s="59" t="inlineStr">
+      <c r="D83" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4463628391/</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="57" t="inlineStr">
+      <c r="A84" s="60" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="B84" s="58" t="n">
+      <c r="B84" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -2320,19 +2329,19 @@
           <t>Sr Business Process Analyst (m/w/d) - Healthcare</t>
         </is>
       </c>
-      <c r="D84" s="59" t="inlineStr">
+      <c r="D84" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4459309508/</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="57" t="inlineStr">
+      <c r="A85" s="60" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="B85" s="58" t="n">
+      <c r="B85" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -2340,19 +2349,19 @@
           <t>Trade Marketing Manager - Pharmacy (m/w/d)</t>
         </is>
       </c>
-      <c r="D85" s="59" t="inlineStr">
+      <c r="D85" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4461770007/</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="57" t="inlineStr">
+      <c r="A86" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B86" s="58" t="n">
+      <c r="B86" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -2360,19 +2369,19 @@
           <t>Associate Territory Sales Manager - Healthcare - Leicestershire &amp; Lincolnshire</t>
         </is>
       </c>
-      <c r="D86" s="59" t="inlineStr">
+      <c r="D86" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453076276/</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="57" t="inlineStr">
+      <c r="A87" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B87" s="58" t="n">
+      <c r="B87" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -2380,19 +2389,19 @@
           <t>Marketing Manager Education Consumer Products EMEA – Healthcare – Bracknell, UK</t>
         </is>
       </c>
-      <c r="D87" s="59" t="inlineStr">
+      <c r="D87" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4462849233/</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="57" t="inlineStr">
+      <c r="A88" s="60" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="B88" s="58" t="n">
+      <c r="B88" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -2400,19 +2409,19 @@
           <t>Sr Manager Regulatory Affairs</t>
         </is>
       </c>
-      <c r="D88" s="59" t="inlineStr">
+      <c r="D88" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4456106944/</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="57" t="inlineStr">
+      <c r="A89" s="60" t="inlineStr">
         <is>
           <t>Ireland</t>
         </is>
       </c>
-      <c r="B89" s="58" t="n">
+      <c r="B89" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -2420,19 +2429,19 @@
           <t>QA Engineer Digital Systems</t>
         </is>
       </c>
-      <c r="D89" s="59" t="inlineStr">
+      <c r="D89" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4444460213/</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="57" t="inlineStr">
+      <c r="A90" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B90" s="58" t="n">
+      <c r="B90" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -2440,19 +2449,19 @@
           <t>Junior Territory Sales Manager - Healthcare - Hertfordshire &amp; Essex</t>
         </is>
       </c>
-      <c r="D90" s="59" t="inlineStr">
+      <c r="D90" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453078274/</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="57" t="inlineStr">
+      <c r="A91" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B91" s="58" t="n">
+      <c r="B91" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -2460,19 +2469,19 @@
           <t>Contract Administration Representative (French-speaking)</t>
         </is>
       </c>
-      <c r="D91" s="59" t="inlineStr">
+      <c r="D91" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4461090763/</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="57" t="inlineStr">
+      <c r="A92" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B92" s="58" t="n">
+      <c r="B92" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -2480,19 +2489,19 @@
           <t>GBS Engagement &amp; Service Management Lead</t>
         </is>
       </c>
-      <c r="D92" s="59" t="inlineStr">
+      <c r="D92" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4427554137/</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="57" t="inlineStr">
+      <c r="A93" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B93" s="58" t="n">
+      <c r="B93" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C93" s="4" t="inlineStr">
@@ -2500,19 +2509,19 @@
           <t>Senior Forecasting Analyst – Healthcare - UK</t>
         </is>
       </c>
-      <c r="D93" s="59" t="inlineStr">
+      <c r="D93" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4463622979/</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="57" t="inlineStr">
+      <c r="A94" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B94" s="58" t="n">
+      <c r="B94" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -2520,19 +2529,19 @@
           <t>Junior Territory Sales Manager - Healthcare - Hertfordshire &amp; Essex</t>
         </is>
       </c>
-      <c r="D94" s="59" t="inlineStr">
+      <c r="D94" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453089165/</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="57" t="inlineStr">
+      <c r="A95" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B95" s="58" t="n">
+      <c r="B95" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -2540,19 +2549,19 @@
           <t>Senior Forecasting Analyst – Healthcare - UK</t>
         </is>
       </c>
-      <c r="D95" s="59" t="inlineStr">
+      <c r="D95" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4463634192/</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="57" t="inlineStr">
+      <c r="A96" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B96" s="58" t="n">
+      <c r="B96" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -2560,19 +2569,19 @@
           <t>Junior Territory Sales Manager - Healthcare - Hertfordshire &amp; Essex</t>
         </is>
       </c>
-      <c r="D96" s="59" t="inlineStr">
+      <c r="D96" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453083196/</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="57" t="inlineStr">
+      <c r="A97" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B97" s="58" t="n">
+      <c r="B97" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -2580,19 +2589,19 @@
           <t>Customer Service Representative, French Speaker</t>
         </is>
       </c>
-      <c r="D97" s="59" t="inlineStr">
+      <c r="D97" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4462772822/</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="57" t="inlineStr">
+      <c r="A98" s="60" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="B98" s="58" t="n">
+      <c r="B98" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -2600,19 +2609,19 @@
           <t>Associate Territory Sales Manager - Healthcare - Leicestershire &amp; Lincolnshire</t>
         </is>
       </c>
-      <c r="D98" s="59" t="inlineStr">
+      <c r="D98" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453082209/</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="57" t="inlineStr">
+      <c r="A99" s="60" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="B99" s="58" t="n">
+      <c r="B99" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -2620,19 +2629,19 @@
           <t>Technical Support Representative 2</t>
         </is>
       </c>
-      <c r="D99" s="59" t="inlineStr">
+      <c r="D99" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4438880089/</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="57" t="inlineStr">
+      <c r="A100" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B100" s="58" t="n">
+      <c r="B100" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -2640,19 +2649,19 @@
           <t>Spanish Bilingual Customer Account Support Specialist 2</t>
         </is>
       </c>
-      <c r="D100" s="59" t="inlineStr">
+      <c r="D100" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4458704406/</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="57" t="inlineStr">
+      <c r="A101" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B101" s="58" t="n">
+      <c r="B101" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -2660,19 +2669,19 @@
           <t>Spanish Bilingual TSR</t>
         </is>
       </c>
-      <c r="D101" s="59" t="inlineStr">
+      <c r="D101" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4407814543/</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="57" t="inlineStr">
+      <c r="A102" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B102" s="58" t="n">
+      <c r="B102" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -2680,19 +2689,19 @@
           <t>Senior Medical Affairs Manager – Value, Evidence, and Outcomes</t>
         </is>
       </c>
-      <c r="D102" s="59" t="inlineStr">
+      <c r="D102" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4443448275/</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="57" t="inlineStr">
+      <c r="A103" s="60" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B103" s="58" t="n">
+      <c r="B103" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -2700,19 +2709,19 @@
           <t>Sr Technical Writer</t>
         </is>
       </c>
-      <c r="D103" s="59" t="inlineStr">
+      <c r="D103" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4465024024/</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="57" t="inlineStr">
+      <c r="A104" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B104" s="58" t="n">
+      <c r="B104" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -2720,19 +2729,19 @@
           <t>Production Chemist 3</t>
         </is>
       </c>
-      <c r="D104" s="59" t="inlineStr">
+      <c r="D104" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4464932915/</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="57" t="inlineStr">
+      <c r="A105" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B105" s="58" t="n">
+      <c r="B105" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -2740,19 +2749,19 @@
           <t>Lead Corporate Development Manager</t>
         </is>
       </c>
-      <c r="D105" s="59" t="inlineStr">
+      <c r="D105" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4462460922/</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="57" t="inlineStr">
+      <c r="A106" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B106" s="58" t="n">
+      <c r="B106" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -2760,19 +2769,19 @@
           <t>Staff QA Engineer</t>
         </is>
       </c>
-      <c r="D106" s="59" t="inlineStr">
+      <c r="D106" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4439353245/</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="57" t="inlineStr">
+      <c r="A107" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B107" s="58" t="n">
+      <c r="B107" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -2780,19 +2789,19 @@
           <t>HR Business Partner</t>
         </is>
       </c>
-      <c r="D107" s="59" t="inlineStr">
+      <c r="D107" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4456322164/</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="57" t="inlineStr">
+      <c r="A108" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B108" s="58" t="n">
+      <c r="B108" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -2800,19 +2809,19 @@
           <t>Procurement Ops Manager (IC)</t>
         </is>
       </c>
-      <c r="D108" s="59" t="inlineStr">
+      <c r="D108" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4453082223/</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="57" t="inlineStr">
+      <c r="A109" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B109" s="58" t="n">
+      <c r="B109" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -2820,19 +2829,19 @@
           <t>Business Process Analyst</t>
         </is>
       </c>
-      <c r="D109" s="59" t="inlineStr">
+      <c r="D109" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4414569192/</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="57" t="inlineStr">
+      <c r="A110" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B110" s="58" t="n">
+      <c r="B110" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C110" s="4" t="inlineStr">
@@ -2840,19 +2849,19 @@
           <t>Sr. Director, Consumer Software Applications</t>
         </is>
       </c>
-      <c r="D110" s="59" t="inlineStr">
+      <c r="D110" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4456380639/</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="57" t="inlineStr">
+      <c r="A111" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B111" s="58" t="n">
+      <c r="B111" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C111" s="4" t="inlineStr">
@@ -2860,19 +2869,19 @@
           <t>Sr. Director, Consumer Software Applications</t>
         </is>
       </c>
-      <c r="D111" s="59" t="inlineStr">
+      <c r="D111" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4456364824/</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="57" t="inlineStr">
+      <c r="A112" s="60" t="inlineStr">
         <is>
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="B112" s="58" t="n">
+      <c r="B112" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C112" s="4" t="inlineStr">
@@ -2880,19 +2889,19 @@
           <t>Associate Marketing Manager</t>
         </is>
       </c>
-      <c r="D112" s="59" t="inlineStr">
+      <c r="D112" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4451399530/</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="57" t="inlineStr">
+      <c r="A113" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B113" s="58" t="n">
+      <c r="B113" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C113" s="4" t="inlineStr">
@@ -2900,19 +2909,19 @@
           <t>Material Handler 1 ( RDC ) - Days 1A and 1B</t>
         </is>
       </c>
-      <c r="D113" s="59" t="inlineStr">
+      <c r="D113" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4455128356/</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="57" t="inlineStr">
+      <c r="A114" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B114" s="58" t="n">
+      <c r="B114" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C114" s="4" t="inlineStr">
@@ -2920,19 +2929,19 @@
           <t>Material Handler 4 ( 2B Thur-Sat, every other Wednesday, Can work anytime from 5pm-5am )</t>
         </is>
       </c>
-      <c r="D114" s="59" t="inlineStr">
+      <c r="D114" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4464432288/</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="57" t="inlineStr">
+      <c r="A115" s="60" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B115" s="58" t="n">
+      <c r="B115" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C115" s="4" t="inlineStr">
@@ -2940,19 +2949,19 @@
           <t>Senior Sterilization Engineer</t>
         </is>
       </c>
-      <c r="D115" s="59" t="inlineStr">
+      <c r="D115" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4410980549/</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="57" t="inlineStr">
+      <c r="A116" s="60" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B116" s="58" t="n">
+      <c r="B116" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C116" s="4" t="inlineStr">
@@ -2960,19 +2969,19 @@
           <t>Accounts Payable Process Expert (Maternity Cover)</t>
         </is>
       </c>
-      <c r="D116" s="59" t="inlineStr">
+      <c r="D116" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4462464542/</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="57" t="inlineStr">
+      <c r="A117" s="60" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B117" s="58" t="n">
+      <c r="B117" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C117" s="4" t="inlineStr">
@@ -2980,19 +2989,19 @@
           <t>Staff Software Test Development Engineer</t>
         </is>
       </c>
-      <c r="D117" s="59" t="inlineStr">
+      <c r="D117" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4388377406/</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="57" t="inlineStr">
+      <c r="A118" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B118" s="58" t="n">
+      <c r="B118" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C118" s="4" t="inlineStr">
@@ -3000,19 +3009,19 @@
           <t>Manager Quality Compliance</t>
         </is>
       </c>
-      <c r="D118" s="59" t="inlineStr">
+      <c r="D118" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4464662874/</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="57" t="inlineStr">
+      <c r="A119" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B119" s="58" t="n">
+      <c r="B119" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C119" s="4" t="inlineStr">
@@ -3020,19 +3029,19 @@
           <t>QA Engineer 2</t>
         </is>
       </c>
-      <c r="D119" s="59" t="inlineStr">
+      <c r="D119" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4464097498/</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="57" t="inlineStr">
+      <c r="A120" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B120" s="58" t="n">
+      <c r="B120" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C120" s="4" t="inlineStr">
@@ -3040,19 +3049,19 @@
           <t>Staff QA Engineer</t>
         </is>
       </c>
-      <c r="D120" s="59" t="inlineStr">
+      <c r="D120" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4436409441/</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="57" t="inlineStr">
+      <c r="A121" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B121" s="58" t="n">
+      <c r="B121" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C121" s="4" t="inlineStr">
@@ -3060,19 +3069,19 @@
           <t>Staff Equipment Engineer</t>
         </is>
       </c>
-      <c r="D121" s="59" t="inlineStr">
+      <c r="D121" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4455253909/</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="57" t="inlineStr">
+      <c r="A122" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B122" s="58" t="n">
+      <c r="B122" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C122" s="4" t="inlineStr">
@@ -3080,19 +3089,19 @@
           <t>Sr. Staff Technical Program Manager - Stelo</t>
         </is>
       </c>
-      <c r="D122" s="59" t="inlineStr">
+      <c r="D122" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4455370480/</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="57" t="inlineStr">
+      <c r="A123" s="60" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B123" s="58" t="n">
+      <c r="B123" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C123" s="4" t="inlineStr">
@@ -3100,19 +3109,19 @@
           <t>Staff SRE SW Development Engineer</t>
         </is>
       </c>
-      <c r="D123" s="59" t="inlineStr">
+      <c r="D123" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4387683946/</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="57" t="inlineStr">
+      <c r="A124" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B124" s="58" t="n">
+      <c r="B124" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C124" s="4" t="inlineStr">
@@ -3120,19 +3129,19 @@
           <t>Material Handler 2 ( RDC ) - Days 1A and 1B</t>
         </is>
       </c>
-      <c r="D124" s="59" t="inlineStr">
+      <c r="D124" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4455289757/</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="57" t="inlineStr">
+      <c r="A125" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B125" s="58" t="n">
+      <c r="B125" s="61" t="n">
         <v>46275</v>
       </c>
       <c r="C125" s="4" t="inlineStr">
@@ -3140,19 +3149,19 @@
           <t>Material Handler 2 ( RDC ) - Nights 2A and 2B</t>
         </is>
       </c>
-      <c r="D125" s="59" t="inlineStr">
+      <c r="D125" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4455289751/</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="57" t="inlineStr">
+      <c r="A126" s="60" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
-      <c r="B126" s="58" t="n">
+      <c r="B126" s="61" t="n">
         <v>46276</v>
       </c>
       <c r="C126" s="4" t="inlineStr">
@@ -3160,369 +3169,369 @@
           <t>Third Party Risk and Supplier Onboarding Manager</t>
         </is>
       </c>
-      <c r="D126" s="59" t="inlineStr">
+      <c r="D126" s="62" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4466048486/</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="57" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="B127" s="58" t="n">
-        <v>46270</v>
+      <c r="A127" s="60" t="inlineStr">
+        <is>
+          <t>Lithuania</t>
+        </is>
+      </c>
+      <c r="B127" s="61" t="n">
+        <v>46274</v>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>Distributor Manager - Channel Excellence (MedTech)</t>
-        </is>
-      </c>
-      <c r="D127" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4463683762/</t>
+          <t>Senior Service Designer, Technical Support</t>
+        </is>
+      </c>
+      <c r="D127" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4455960251/</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="57" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="B128" s="58" t="n">
-        <v>46270</v>
+      <c r="A128" s="60" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="B128" s="61" t="n">
+        <v>46273</v>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>Distributor Manager - Channel Excellence (MedTech)</t>
-        </is>
-      </c>
-      <c r="D128" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4463684766/</t>
+          <t>Process Technician 2 (Front End Night Shift)</t>
+        </is>
+      </c>
+      <c r="D128" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4455755200/</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="57" t="inlineStr">
-        <is>
-          <t>Lithuania</t>
-        </is>
-      </c>
-      <c r="B129" s="58" t="n">
+      <c r="A129" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B129" s="61" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t>Manager Systems Design Engineering</t>
+        </is>
+      </c>
+      <c r="D129" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4464683405/</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B130" s="61" t="n">
         <v>46274</v>
       </c>
-      <c r="C129" s="4" t="inlineStr">
-        <is>
-          <t>Senior Service Designer, Technical Support</t>
-        </is>
-      </c>
-      <c r="D129" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4455960251/</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="57" t="inlineStr">
-        <is>
-          <t>Ireland</t>
-        </is>
-      </c>
-      <c r="B130" s="58" t="n">
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>Senior Staff Process Development Engineer</t>
+        </is>
+      </c>
+      <c r="D130" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4464945232/</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="60" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B131" s="61" t="n">
         <v>46273</v>
       </c>
-      <c r="C130" s="4" t="inlineStr">
-        <is>
-          <t>Process Technician 2 (Front End Night Shift)</t>
-        </is>
-      </c>
-      <c r="D130" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4455755200/</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="57" t="inlineStr">
-        <is>
-          <t>Ireland</t>
-        </is>
-      </c>
-      <c r="B131" s="58" t="n">
-        <v>46272</v>
-      </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Supervisor Process Engineering</t>
-        </is>
-      </c>
-      <c r="D131" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4464338496/</t>
+          <t>Manager, SW System &amp; Solution Dev Engineer</t>
+        </is>
+      </c>
+      <c r="D131" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4464452799/</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="57" t="inlineStr">
-        <is>
-          <t>Ireland</t>
-        </is>
-      </c>
-      <c r="B132" s="58" t="n">
-        <v>46272</v>
+      <c r="A132" s="60" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="B132" s="61" t="n">
+        <v>46274</v>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Sr Production Supervisor (Front End Night Shift)</t>
-        </is>
-      </c>
-      <c r="D132" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4455302580/</t>
+          <t>Supervisor Manufacturing</t>
+        </is>
+      </c>
+      <c r="D132" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4428861138/</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="57" t="inlineStr">
-        <is>
-          <t>Ireland</t>
-        </is>
-      </c>
-      <c r="B133" s="58" t="n">
-        <v>46270</v>
+      <c r="A133" s="60" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="B133" s="61" t="n">
+        <v>46274</v>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Engineering Technician 3 (Front End Day Shift)</t>
-        </is>
-      </c>
-      <c r="D133" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4463698028/</t>
+          <t>Staff Database Administrator</t>
+        </is>
+      </c>
+      <c r="D133" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4456322200/</t>
         </is>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="57" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-      <c r="B134" s="58" t="n">
-        <v>46272</v>
+      <c r="A134" s="60" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="B134" s="61" t="n">
+        <v>46274</v>
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Territory Business Manager</t>
-        </is>
-      </c>
-      <c r="D134" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4464350389/</t>
+          <t>Payroll Analyst (ANZ)</t>
+        </is>
+      </c>
+      <c r="D134" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4456178209/</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="57" t="inlineStr">
+      <c r="A135" s="60" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="B135" s="61" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>Sr Enterprise Developer (Power Platform Developer)</t>
+        </is>
+      </c>
+      <c r="D135" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4455767052/</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B135" s="58" t="n">
+      <c r="B136" s="61" t="n">
         <v>46273</v>
       </c>
-      <c r="C135" s="4" t="inlineStr">
-        <is>
-          <t>Manager Systems Design Engineering</t>
-        </is>
-      </c>
-      <c r="D135" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4464683405/</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="57" t="inlineStr">
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>Software QA Engineer 2</t>
+        </is>
+      </c>
+      <c r="D136" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4464606837/</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="60" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B137" s="61" t="n">
+        <v>46274</v>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>SW Test Development Engineer 1</t>
+        </is>
+      </c>
+      <c r="D137" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4465029007/</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="60" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B138" s="61" t="n">
+        <v>46273</v>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>SW Development Engineer 2 - Android</t>
+        </is>
+      </c>
+      <c r="D138" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4464610755/</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B136" s="58" t="n">
+      <c r="B139" s="61" t="n">
         <v>46274</v>
       </c>
-      <c r="C136" s="4" t="inlineStr">
-        <is>
-          <t>Senior Staff Process Development Engineer</t>
-        </is>
-      </c>
-      <c r="D136" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4464945232/</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="57" t="inlineStr">
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>Sr Workplace Solutions Analyst</t>
+        </is>
+      </c>
+      <c r="D139" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4456322161/</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="60" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B137" s="58" t="n">
-        <v>46273</v>
-      </c>
-      <c r="C137" s="4" t="inlineStr">
-        <is>
-          <t>Manager, SW System &amp; Solution Dev Engineer</t>
-        </is>
-      </c>
-      <c r="D137" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4464452799/</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="57" t="inlineStr">
+      <c r="B140" s="61" t="n">
+        <v>46274</v>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>Staff SW Development Engineer</t>
+        </is>
+      </c>
+      <c r="D140" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4465323573/</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="60" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="B141" s="61" t="n">
+        <v>46274</v>
+      </c>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>Director, Business Program Management Office</t>
+        </is>
+      </c>
+      <c r="D141" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4456105988/</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="60" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="B138" s="58" t="n">
+      <c r="B142" s="61" t="n">
         <v>46274</v>
       </c>
-      <c r="C138" s="4" t="inlineStr">
-        <is>
-          <t>Supervisor Manufacturing</t>
-        </is>
-      </c>
-      <c r="D138" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4428861138/</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="57" t="inlineStr">
-        <is>
-          <t>Malaysia</t>
-        </is>
-      </c>
-      <c r="B139" s="58" t="n">
-        <v>46270</v>
-      </c>
-      <c r="C139" s="4" t="inlineStr">
-        <is>
-          <t>Sr IT Project Manager</t>
-        </is>
-      </c>
-      <c r="D139" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4436188818/</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="57" t="inlineStr">
-        <is>
-          <t>Philippines</t>
-        </is>
-      </c>
-      <c r="B140" s="58" t="n">
+      <c r="C142" s="4" t="inlineStr">
+        <is>
+          <t>Engineering Technician 4</t>
+        </is>
+      </c>
+      <c r="D142" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4456115187/</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B143" s="61" t="n">
         <v>46274</v>
       </c>
-      <c r="C140" s="4" t="inlineStr">
-        <is>
-          <t>Staff Database Administrator</t>
-        </is>
-      </c>
-      <c r="D140" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4456322200/</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="57" t="inlineStr">
-        <is>
-          <t>Philippines</t>
-        </is>
-      </c>
-      <c r="B141" s="58" t="n">
-        <v>46274</v>
-      </c>
-      <c r="C141" s="4" t="inlineStr">
-        <is>
-          <t>Payroll Analyst (ANZ)</t>
-        </is>
-      </c>
-      <c r="D141" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4456178209/</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="57" t="inlineStr">
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>Systems Design &amp; Test Engineer 2</t>
+        </is>
+      </c>
+      <c r="D143" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4443989564/</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="60" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B142" s="58" t="n">
-        <v>46270</v>
-      </c>
-      <c r="C142" s="4" t="inlineStr">
-        <is>
-          <t>Senior Staff Mechanical Engineer - Characterization Lead</t>
-        </is>
-      </c>
-      <c r="D142" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4427645063/</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="57" t="inlineStr">
-        <is>
-          <t>Philippines</t>
-        </is>
-      </c>
-      <c r="B143" s="58" t="n">
-        <v>46273</v>
-      </c>
-      <c r="C143" s="4" t="inlineStr">
-        <is>
-          <t>Sr Enterprise Developer (Power Platform Developer)</t>
-        </is>
-      </c>
-      <c r="D143" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4455767052/</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="57" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="B144" s="58" t="n">
-        <v>46273</v>
+      <c r="B144" s="61" t="n">
+        <v>46275</v>
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>Software QA Engineer 2</t>
-        </is>
-      </c>
-      <c r="D144" s="59" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4464606837/</t>
+          <t>Sr. Staff Technical Program Manager - Sensor Technology</t>
+        </is>
+      </c>
+      <c r="D144" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4439394782/</t>
         </is>
       </c>
     </row>
@@ -3533,261 +3542,701 @@
         </is>
       </c>
       <c r="B145" s="61" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
+          <t>Sr. SW Test Development Engineer V&amp;V</t>
+        </is>
+      </c>
+      <c r="D145" s="62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4387839555/</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="63" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B146" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C146" s="4" t="inlineStr">
+        <is>
           <t>SW Development Engineer 1 - Android</t>
         </is>
       </c>
-      <c r="D145" s="62" t="inlineStr">
+      <c r="D146" s="65" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/jobs/view/4464353380/</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="60" t="inlineStr">
+    <row r="147">
+      <c r="A147" s="63" t="inlineStr">
+        <is>
+          <t>Lithuania</t>
+        </is>
+      </c>
+      <c r="B147" s="64" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>Sr. Financial Analyst</t>
+        </is>
+      </c>
+      <c r="D147" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4421230278/</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="63" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B146" s="61" t="n">
+      <c r="B148" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C148" s="4" t="inlineStr">
+        <is>
+          <t>Sr Cybersecurity Analyst</t>
+        </is>
+      </c>
+      <c r="D148" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4439085443/</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="63" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B149" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>SW Development Engineer 2</t>
+        </is>
+      </c>
+      <c r="D149" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4460357219/</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="63" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="B150" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C150" s="4" t="inlineStr">
+        <is>
+          <t>Trade Compliance Analyst</t>
+        </is>
+      </c>
+      <c r="D150" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4467033928/</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="63" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B151" s="64" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>Sr Manufacturing Engineer</t>
+        </is>
+      </c>
+      <c r="D151" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4447583072/</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="63" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="B152" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C152" s="4" t="inlineStr">
+        <is>
+          <t>Staff Vendor Management Analyst</t>
+        </is>
+      </c>
+      <c r="D152" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4458212554/</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="63" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="B153" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C153" s="4" t="inlineStr">
+        <is>
+          <t>Staff Equipment Engineer</t>
+        </is>
+      </c>
+      <c r="D153" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4458218533/</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="63" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="B154" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C154" s="4" t="inlineStr">
+        <is>
+          <t>APAC Product Manager - OTC/Consumer Health</t>
+        </is>
+      </c>
+      <c r="D154" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4422693615/</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="63" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="B155" s="64" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>Supervisor Technical Support - Manila</t>
+        </is>
+      </c>
+      <c r="D155" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4417742237/</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="63" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="B156" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C156" s="4" t="inlineStr">
+        <is>
+          <t>Staff Desktop Support Engineer</t>
+        </is>
+      </c>
+      <c r="D156" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4398315987/</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="63" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B157" s="64" t="n">
+        <v>46276</v>
+      </c>
+      <c r="C157" s="4" t="inlineStr">
+        <is>
+          <t>Director HW Design Quality Engineering - New Product Introductions</t>
+        </is>
+      </c>
+      <c r="D157" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4456789792/</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="63" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B158" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C158" s="4" t="inlineStr">
+        <is>
+          <t>Manager SW Test Development Engineering</t>
+        </is>
+      </c>
+      <c r="D158" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4281993770/</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="63" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B159" s="64" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C159" s="4" t="inlineStr">
+        <is>
+          <t>Document Control and Training Specialist 1 ( Monday to Friday, 8:00 AM - 5:00 PM )</t>
+        </is>
+      </c>
+      <c r="D159" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4463157831/</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="63" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="B160" s="64" t="n">
         <v>46274</v>
       </c>
-      <c r="C146" s="4" t="inlineStr">
-        <is>
-          <t>SW Test Development Engineer 1</t>
-        </is>
-      </c>
-      <c r="D146" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4465029007/</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="60" t="inlineStr">
+      <c r="C160" s="4" t="inlineStr">
+        <is>
+          <t>Supervisor, Applications Support</t>
+        </is>
+      </c>
+      <c r="D160" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4456333076/</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="63" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B161" s="64" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C161" s="4" t="inlineStr">
+        <is>
+          <t>Hardware Engineer 2</t>
+        </is>
+      </c>
+      <c r="D161" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4454834815/</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="63" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="B162" s="64" t="n">
+        <v>46274</v>
+      </c>
+      <c r="C162" s="4" t="inlineStr">
+        <is>
+          <t>Territory Business Manager - South Island</t>
+        </is>
+      </c>
+      <c r="D162" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4456111920/</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="63" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="B163" s="64" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C163" s="4" t="inlineStr">
+        <is>
+          <t>Sr Staff Program Manager</t>
+        </is>
+      </c>
+      <c r="D163" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4448138066/</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="63" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B164" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C164" s="4" t="inlineStr">
+        <is>
+          <t>Senior Manager- Manufacturing IT Strategic Initiatives and Architecture</t>
+        </is>
+      </c>
+      <c r="D164" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4421221561/</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="63" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="B165" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C165" s="4" t="inlineStr">
+        <is>
+          <t>Manager Process Engineering</t>
+        </is>
+      </c>
+      <c r="D165" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4467096658/</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="63" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B147" s="61" t="n">
-        <v>46273</v>
-      </c>
-      <c r="C147" s="4" t="inlineStr">
-        <is>
-          <t>SW Development Engineer 2 - Android</t>
-        </is>
-      </c>
-      <c r="D147" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4464610755/</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="60" t="inlineStr">
+      <c r="B166" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C166" s="4" t="inlineStr">
+        <is>
+          <t>SW Development Engineer 2 - IOS</t>
+        </is>
+      </c>
+      <c r="D166" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4465306719/</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="63" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B167" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C167" s="4" t="inlineStr">
+        <is>
+          <t>Staff Systems Engineer</t>
+        </is>
+      </c>
+      <c r="D167" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4461770016/</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="63" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B148" s="61" t="n">
+      <c r="B168" s="64" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C168" s="4" t="inlineStr">
+        <is>
+          <t>District Business Manager - Ohio</t>
+        </is>
+      </c>
+      <c r="D168" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4458551771/</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="63" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B169" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C169" s="4" t="inlineStr">
+        <is>
+          <t>Systems Engineer</t>
+        </is>
+      </c>
+      <c r="D169" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4375183129/</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="63" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B170" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C170" s="4" t="inlineStr">
+        <is>
+          <t>Lead Firmware V&amp;V</t>
+        </is>
+      </c>
+      <c r="D170" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4402920307/</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="63" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B171" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C171" s="4" t="inlineStr">
+        <is>
+          <t>Sr. Systems Engineer</t>
+        </is>
+      </c>
+      <c r="D171" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4461756319/</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="63" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B172" s="64" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C172" s="4" t="inlineStr">
+        <is>
+          <t>Senior Lead Government Affairs Manager - Federal</t>
+        </is>
+      </c>
+      <c r="D172" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4440825647/</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="63" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="B173" s="64" t="n">
         <v>46274</v>
       </c>
-      <c r="C148" s="4" t="inlineStr">
-        <is>
-          <t>Sr Workplace Solutions Analyst</t>
-        </is>
-      </c>
-      <c r="D148" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4456322161/</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="60" t="inlineStr">
+      <c r="C173" s="4" t="inlineStr">
+        <is>
+          <t>Staff Database Administrator</t>
+        </is>
+      </c>
+      <c r="D173" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4456333107/</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="63" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B174" s="64" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C174" s="4" t="inlineStr">
+        <is>
+          <t>Equipment Technician 2 (2A Sunday - Tuesday, every other Saturday from 5:00PM - 5:00AM )</t>
+        </is>
+      </c>
+      <c r="D174" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4466467687/</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="63" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B175" s="64" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C175" s="4" t="inlineStr">
+        <is>
+          <t>Equipment Technician 2 (2B Wednesday - Friday, every other Saturday from 5:00PM - 5:00AM)</t>
+        </is>
+      </c>
+      <c r="D175" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4466428944/</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="63" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B176" s="64" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C176" s="4" t="inlineStr">
+        <is>
+          <t>New Business Development Manager, Trade Partnerships (eCommerce)</t>
+        </is>
+      </c>
+      <c r="D176" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4459020959/</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="63" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B149" s="61" t="n">
-        <v>46274</v>
-      </c>
-      <c r="C149" s="4" t="inlineStr">
-        <is>
-          <t>Staff SW Development Engineer</t>
-        </is>
-      </c>
-      <c r="D149" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4465323573/</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="60" t="inlineStr">
-        <is>
-          <t>Philippines</t>
-        </is>
-      </c>
-      <c r="B150" s="61" t="n">
-        <v>46274</v>
-      </c>
-      <c r="C150" s="4" t="inlineStr">
-        <is>
-          <t>Director, Business Program Management Office</t>
-        </is>
-      </c>
-      <c r="D150" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4456105988/</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="60" t="inlineStr">
-        <is>
-          <t>Philippines</t>
-        </is>
-      </c>
-      <c r="B151" s="61" t="n">
-        <v>46272</v>
-      </c>
-      <c r="C151" s="4" t="inlineStr">
-        <is>
-          <t>Desktop Support Specialist 3</t>
-        </is>
-      </c>
-      <c r="D151" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4445930979/</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="60" t="inlineStr">
-        <is>
-          <t>Malaysia</t>
-        </is>
-      </c>
-      <c r="B152" s="61" t="n">
-        <v>46274</v>
-      </c>
-      <c r="C152" s="4" t="inlineStr">
-        <is>
-          <t>Engineering Technician 4</t>
-        </is>
-      </c>
-      <c r="D152" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4456115187/</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="60" t="inlineStr">
+      <c r="B177" s="64" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C177" s="4" t="inlineStr">
+        <is>
+          <t>Sr Firmware V&amp;V</t>
+        </is>
+      </c>
+      <c r="D177" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4402292560/</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="63" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B153" s="61" t="n">
-        <v>46274</v>
-      </c>
-      <c r="C153" s="4" t="inlineStr">
-        <is>
-          <t>Systems Design &amp; Test Engineer 2</t>
-        </is>
-      </c>
-      <c r="D153" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4443989564/</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="60" t="inlineStr">
+      <c r="B178" s="64" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C178" s="4" t="inlineStr">
+        <is>
+          <t>Sr Software QA Engineer</t>
+        </is>
+      </c>
+      <c r="D178" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4457557361/</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="63" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="B154" s="61" t="n">
-        <v>46275</v>
-      </c>
-      <c r="C154" s="4" t="inlineStr">
-        <is>
-          <t>Sr. Staff Technical Program Manager - Sensor Technology</t>
-        </is>
-      </c>
-      <c r="D154" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4439394782/</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="60" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="B155" s="61" t="n">
-        <v>46273</v>
-      </c>
-      <c r="C155" s="4" t="inlineStr">
-        <is>
-          <t>Sr. SW Test Development Engineer V&amp;V</t>
-        </is>
-      </c>
-      <c r="D155" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4387839555/</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="60" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="B156" s="61" t="n">
-        <v>46270</v>
-      </c>
-      <c r="C156" s="4" t="inlineStr">
-        <is>
-          <t>QA Inspector 2 ( Dobson ) - 1A Sun- Tues, every other Wednesday, Can work anytime from 5am-5pm</t>
-        </is>
-      </c>
-      <c r="D156" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4463691655/</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="60" t="inlineStr">
-        <is>
-          <t>Ireland</t>
-        </is>
-      </c>
-      <c r="B157" s="61" t="n">
-        <v>46272</v>
-      </c>
-      <c r="C157" s="4" t="inlineStr">
-        <is>
-          <t>Lab Technician 3 (Chemistry) Back End Days</t>
-        </is>
-      </c>
-      <c r="D157" s="62" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4464341469/</t>
+      <c r="B179" s="64" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C179" s="4" t="inlineStr">
+        <is>
+          <t>Staff Enterprise Applications Developer - IBM Maximo</t>
+        </is>
+      </c>
+      <c r="D179" s="65" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4411935028/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D157"/>
+  <autoFilter ref="A1:D179"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -3945,6 +4394,28 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D155" r:id="rId154"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D156" r:id="rId155"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D179" r:id="rId178"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>